<commit_message>
chore: consolidate project updates
</commit_message>
<xml_diff>
--- a/nav/润洲正行11号私募证券投资基金A_净值序列_20250506.xlsx
+++ b/nav/润洲正行11号私募证券投资基金A_净值序列_20250506.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/190c05429d74bb0c/Desktop/nav/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\shaw\yungu\nav\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{F0572404-95CD-48EE-B893-84B18DD40262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4DFF005-FDE8-4139-9893-45B8807DA0AD}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F86A102-A612-4D8D-ACE0-0EFAEF36F8E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1536" yWindow="1536" windowWidth="23040" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-444" yWindow="228" windowWidth="18888" windowHeight="15228" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
@@ -4421,7 +4421,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G623"/>
+  <dimension ref="A1:G641"/>
   <sheetFormatPr defaultColWidth="21" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="16.44140625" customWidth="1"/>
@@ -16535,11 +16535,11 @@
         <v>1.5490999999999999</v>
       </c>
       <c r="F601" s="4">
-        <f t="shared" ref="F601:F623" si="13">E601/$E$402-1</f>
+        <f t="shared" ref="F601:F640" si="13">E601/$E$402-1</f>
         <v>5.3379572963416333E-2</v>
       </c>
       <c r="G601" s="5">
-        <f t="shared" ref="G601:G623" si="14">E601/$E$327-1</f>
+        <f t="shared" ref="G601:G640" si="14">E601/$E$327-1</f>
         <v>0.18278995189738101</v>
       </c>
     </row>
@@ -17092,6 +17092,332 @@
         <f t="shared" si="14"/>
         <v>0.10460410781094898</v>
       </c>
+    </row>
+    <row r="624" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C624" s="2">
+        <v>46108</v>
+      </c>
+      <c r="D624">
+        <v>0.89529999999999998</v>
+      </c>
+      <c r="E624">
+        <v>1.4516</v>
+      </c>
+      <c r="F624" s="3">
+        <f t="shared" si="13"/>
+        <v>-1.2919896640826822E-2</v>
+      </c>
+      <c r="G624" s="5">
+        <f t="shared" si="14"/>
+        <v>0.10834542261586622</v>
+      </c>
+    </row>
+    <row r="625" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C625" s="2">
+        <v>46111</v>
+      </c>
+      <c r="D625">
+        <v>0.89070000000000005</v>
+      </c>
+      <c r="E625">
+        <v>1.4470000000000001</v>
+      </c>
+      <c r="F625" s="3">
+        <f t="shared" si="13"/>
+        <v>-1.6047871617026921E-2</v>
+      </c>
+      <c r="G625" s="5">
+        <f t="shared" si="14"/>
+        <v>0.10483316790104591</v>
+      </c>
+    </row>
+    <row r="626" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C626" s="2">
+        <v>46112</v>
+      </c>
+      <c r="D626">
+        <v>0.91879999999999995</v>
+      </c>
+      <c r="E626">
+        <v>1.4751000000000001</v>
+      </c>
+      <c r="F626" s="3">
+        <f t="shared" si="13"/>
+        <v>3.0599755201958789E-3</v>
+      </c>
+      <c r="G626" s="5">
+        <f t="shared" si="14"/>
+        <v>0.12628846300679553</v>
+      </c>
+    </row>
+    <row r="627" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C627" s="2">
+        <v>46113</v>
+      </c>
+      <c r="D627">
+        <v>0.94069999999999998</v>
+      </c>
+      <c r="E627">
+        <v>1.4970000000000001</v>
+      </c>
+      <c r="F627" s="3">
+        <f t="shared" si="13"/>
+        <v>1.7951856385149068E-2</v>
+      </c>
+      <c r="G627" s="5">
+        <f t="shared" si="14"/>
+        <v>0.14300984958387408</v>
+      </c>
+    </row>
+    <row r="628" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C628" s="2">
+        <v>46114</v>
+      </c>
+      <c r="D628">
+        <v>0.93340000000000001</v>
+      </c>
+      <c r="E628">
+        <v>1.4897</v>
+      </c>
+      <c r="F628" s="3">
+        <f t="shared" si="13"/>
+        <v>1.2987896096831264E-2</v>
+      </c>
+      <c r="G628" s="5">
+        <f t="shared" si="14"/>
+        <v>0.13743605405818116</v>
+      </c>
+    </row>
+    <row r="629" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C629" s="2">
+        <v>46115</v>
+      </c>
+      <c r="D629">
+        <v>0.93520000000000003</v>
+      </c>
+      <c r="E629">
+        <v>1.4915</v>
+      </c>
+      <c r="F629" s="3">
+        <f t="shared" si="13"/>
+        <v>1.421188630490966E-2</v>
+      </c>
+      <c r="G629" s="5">
+        <f t="shared" si="14"/>
+        <v>0.13881041459876298</v>
+      </c>
+    </row>
+    <row r="630" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C630" s="2">
+        <v>46119</v>
+      </c>
+      <c r="D630">
+        <v>0.93600000000000005</v>
+      </c>
+      <c r="E630">
+        <v>1.4923</v>
+      </c>
+      <c r="F630" s="3">
+        <f t="shared" si="13"/>
+        <v>1.4755881952944305E-2</v>
+      </c>
+      <c r="G630" s="5">
+        <f t="shared" si="14"/>
+        <v>0.13942124150568813</v>
+      </c>
+    </row>
+    <row r="631" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C631" s="2">
+        <v>46120</v>
+      </c>
+      <c r="D631">
+        <v>0.93110000000000004</v>
+      </c>
+      <c r="E631">
+        <v>1.4874000000000001</v>
+      </c>
+      <c r="F631" s="3">
+        <f t="shared" si="13"/>
+        <v>1.1423908608731326E-2</v>
+      </c>
+      <c r="G631" s="5">
+        <f t="shared" si="14"/>
+        <v>0.13567992670077111</v>
+      </c>
+    </row>
+    <row r="632" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C632" s="2">
+        <v>46121</v>
+      </c>
+      <c r="D632">
+        <v>0.92849999999999999</v>
+      </c>
+      <c r="E632">
+        <v>1.4847999999999999</v>
+      </c>
+      <c r="F632" s="3">
+        <f t="shared" si="13"/>
+        <v>9.6559227526180624E-3</v>
+      </c>
+      <c r="G632" s="5">
+        <f t="shared" si="14"/>
+        <v>0.13369473925326392</v>
+      </c>
+    </row>
+    <row r="633" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C633" s="2">
+        <v>46122</v>
+      </c>
+      <c r="D633">
+        <v>0.93630000000000002</v>
+      </c>
+      <c r="E633">
+        <v>1.4925999999999999</v>
+      </c>
+      <c r="F633" s="3">
+        <f t="shared" si="13"/>
+        <v>1.4959880320957408E-2</v>
+      </c>
+      <c r="G633" s="5">
+        <f t="shared" si="14"/>
+        <v>0.13965030159578506</v>
+      </c>
+    </row>
+    <row r="634" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C634" s="2">
+        <v>46125</v>
+      </c>
+      <c r="D634">
+        <v>0.92759999999999998</v>
+      </c>
+      <c r="E634">
+        <v>1.4839</v>
+      </c>
+      <c r="F634" s="3">
+        <f t="shared" si="13"/>
+        <v>9.0439276485789755E-3</v>
+      </c>
+      <c r="G634" s="5">
+        <f t="shared" si="14"/>
+        <v>0.13300755898297312</v>
+      </c>
+    </row>
+    <row r="635" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C635" s="2">
+        <v>46126</v>
+      </c>
+      <c r="D635">
+        <v>0.93969999999999998</v>
+      </c>
+      <c r="E635">
+        <v>1.496</v>
+      </c>
+      <c r="F635" s="3">
+        <f t="shared" si="13"/>
+        <v>1.7271861825105539E-2</v>
+      </c>
+      <c r="G635" s="5">
+        <f t="shared" si="14"/>
+        <v>0.14224631595021764</v>
+      </c>
+    </row>
+    <row r="636" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C636" s="2">
+        <v>46127</v>
+      </c>
+      <c r="D636">
+        <v>0.94389999999999996</v>
+      </c>
+      <c r="E636">
+        <v>1.5002</v>
+      </c>
+      <c r="F636" s="3">
+        <f t="shared" si="13"/>
+        <v>2.0127838977288315E-2</v>
+      </c>
+      <c r="G636" s="5">
+        <f t="shared" si="14"/>
+        <v>0.14545315721157515</v>
+      </c>
+    </row>
+    <row r="637" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C637" s="2">
+        <v>46128</v>
+      </c>
+      <c r="D637">
+        <v>0.95709999999999995</v>
+      </c>
+      <c r="E637">
+        <v>1.5134000000000001</v>
+      </c>
+      <c r="F637" s="3">
+        <f t="shared" si="13"/>
+        <v>2.9103767169862849E-2</v>
+      </c>
+      <c r="G637" s="5">
+        <f t="shared" si="14"/>
+        <v>0.15553180117584176</v>
+      </c>
+    </row>
+    <row r="638" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C638" s="2">
+        <v>46129</v>
+      </c>
+      <c r="D638">
+        <v>0.95860000000000001</v>
+      </c>
+      <c r="E638">
+        <v>1.5148999999999999</v>
+      </c>
+      <c r="F638" s="3">
+        <f t="shared" si="13"/>
+        <v>3.012375900992792E-2</v>
+      </c>
+      <c r="G638" s="5">
+        <f t="shared" si="14"/>
+        <v>0.15667710162632642</v>
+      </c>
+    </row>
+    <row r="639" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C639" s="2">
+        <v>46132</v>
+      </c>
+      <c r="D639">
+        <v>0.97030000000000005</v>
+      </c>
+      <c r="E639">
+        <v>1.5266</v>
+      </c>
+      <c r="F639" s="3">
+        <f t="shared" si="13"/>
+        <v>3.807969536243716E-2</v>
+      </c>
+      <c r="G639" s="5">
+        <f t="shared" si="14"/>
+        <v>0.16561044514010836</v>
+      </c>
+    </row>
+    <row r="640" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C640" s="2">
+        <v>46133</v>
+      </c>
+      <c r="D640">
+        <v>0.96789999999999998</v>
+      </c>
+      <c r="E640">
+        <v>1.5242</v>
+      </c>
+      <c r="F640" s="3">
+        <f t="shared" si="13"/>
+        <v>3.644770841833278E-2</v>
+      </c>
+      <c r="G640" s="5">
+        <f t="shared" si="14"/>
+        <v>0.16377796441933268</v>
+      </c>
+    </row>
+    <row r="641" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C641" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>